<commit_message>
security: remove exposed credentials and harden source code
- Delete diagnostic.ts, check_db.js, check_final.ts, check_sri_status.ts
  (contained hardcoded Supabase service_role JWT — GitHub secret alert)
- Delete Prompt.txt and Restaurantes Prompt y Desarrollo.txt
  (contained plaintext passwords and email credentials)
- Remove hardcoded fallback keys from all supabase.ts files
  (QI, VendorManagement, LedgerPro, Importaciones now require env vars)
- Exclude App/Proyecto Restaurantes (embedded git repo)
- Update .gitignore to block debug scripts, prompt files and .venv

ACTION REQUIRED: Rotate the Supabase service_role key for project
alttjjytmcrixghxavbt — it was exposed in git history since commit 5f45a71c

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/App/Ledger Pro/Plantilla Ventas Externas.xlsx
+++ b/App/Ledger Pro/Plantilla Ventas Externas.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1514" uniqueCount="380">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1516" uniqueCount="383">
   <si>
     <t/>
   </si>
@@ -1123,9 +1123,6 @@
     <t>valor IVA</t>
   </si>
   <si>
-    <t>Retencion en la Fuente</t>
-  </si>
-  <si>
     <t>base</t>
   </si>
   <si>
@@ -1135,12 +1132,6 @@
     <t>Valor</t>
   </si>
   <si>
-    <t>Retencion Transporte</t>
-  </si>
-  <si>
-    <t>Retencion IVA</t>
-  </si>
-  <si>
     <t>Base Iva 0%</t>
   </si>
   <si>
@@ -1150,23 +1141,41 @@
     <t>Base Iva 15%</t>
   </si>
   <si>
-    <t>Cedulaa/Ruc</t>
-  </si>
-  <si>
-    <t>Tasa IVA</t>
-  </si>
-  <si>
     <t>Total Bases</t>
   </si>
   <si>
     <t>importe Total</t>
+  </si>
+  <si>
+    <t>efectivo</t>
+  </si>
+  <si>
+    <t>cheques</t>
+  </si>
+  <si>
+    <t>transferencias</t>
+  </si>
+  <si>
+    <t>otros</t>
+  </si>
+  <si>
+    <t>Estab</t>
+  </si>
+  <si>
+    <t>Cedula/Ruc</t>
+  </si>
+  <si>
+    <t>crédito</t>
+  </si>
+  <si>
+    <t>tarjetas</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -1195,6 +1204,11 @@
       <sz val="12"/>
       <color theme="0"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -1274,7 +1288,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1282,13 +1296,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="2" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1309,6 +1317,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1613,7 +1622,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Z2"/>
+  <dimension ref="A1:AE1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -1624,19 +1633,20 @@
     <col min="7" max="7" width="14.85546875" customWidth="1"/>
     <col min="8" max="8" width="15.28515625" customWidth="1"/>
     <col min="9" max="9" width="14.28515625" customWidth="1"/>
-    <col min="11" max="11" width="14.5703125" customWidth="1"/>
-    <col min="12" max="12" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10" style="8" bestFit="1" customWidth="1"/>
-    <col min="15" max="26" width="9.140625" style="8"/>
+    <col min="10" max="10" width="14.5703125" customWidth="1"/>
+    <col min="11" max="11" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="18" width="13.85546875" customWidth="1"/>
+    <col min="19" max="19" width="10" style="7" bestFit="1" customWidth="1"/>
+    <col min="20" max="31" width="9.140625" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="15.75">
+    <row r="1" spans="1:27" ht="15.75">
       <c r="A1" s="3" t="s">
         <v>1</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>2</v>
+        <v>379</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>3</v>
@@ -1647,94 +1657,74 @@
       <c r="E1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="14" t="s">
+        <v>380</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>370</v>
+      </c>
+      <c r="H1" s="10" t="s">
+        <v>371</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>372</v>
+      </c>
+      <c r="J1" s="12" t="s">
+        <v>373</v>
+      </c>
+      <c r="K1" s="12" t="s">
+        <v>366</v>
+      </c>
+      <c r="L1" s="13" t="s">
+        <v>374</v>
+      </c>
+      <c r="M1" s="13" t="s">
+        <v>375</v>
+      </c>
+      <c r="N1" s="14" t="s">
+        <v>381</v>
+      </c>
+      <c r="O1" s="13" t="s">
         <v>376</v>
       </c>
-      <c r="G1" s="12" t="s">
-        <v>373</v>
-      </c>
-      <c r="H1" s="12" t="s">
-        <v>374</v>
-      </c>
-      <c r="I1" s="13" t="s">
-        <v>375</v>
-      </c>
-      <c r="J1" s="14" t="s">
+      <c r="P1" s="13" t="s">
         <v>377</v>
       </c>
-      <c r="K1" s="14" t="s">
+      <c r="Q1" s="14" t="s">
+        <v>382</v>
+      </c>
+      <c r="R1" s="13" t="s">
         <v>378</v>
       </c>
-      <c r="L1" s="14" t="s">
-        <v>366</v>
-      </c>
-      <c r="M1" s="15" t="s">
-        <v>379</v>
-      </c>
-      <c r="N1" s="9" t="s">
+      <c r="S1" s="8" t="s">
         <v>367</v>
       </c>
-      <c r="O1" s="9"/>
-      <c r="P1" s="9"/>
-      <c r="Q1" s="9" t="s">
-        <v>371</v>
-      </c>
-      <c r="R1" s="9"/>
-      <c r="S1" s="9"/>
-      <c r="T1" s="9" t="s">
-        <v>372</v>
-      </c>
-      <c r="U1" s="9"/>
-      <c r="V1" s="9"/>
-    </row>
-    <row r="2" spans="1:22" ht="15.75">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="13"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="14"/>
-      <c r="L2" s="14"/>
-      <c r="M2" s="15"/>
-      <c r="N2" s="10" t="s">
+      <c r="T1" s="8" t="s">
         <v>368</v>
       </c>
-      <c r="O2" s="10" t="s">
+      <c r="U1" s="9" t="s">
         <v>369</v>
       </c>
-      <c r="P2" s="11" t="s">
-        <v>370</v>
-      </c>
-      <c r="Q2" s="10" t="s">
+      <c r="V1" s="8" t="s">
+        <v>367</v>
+      </c>
+      <c r="W1" s="8" t="s">
         <v>368</v>
       </c>
-      <c r="R2" s="10" t="s">
+      <c r="X1" s="9" t="s">
         <v>369</v>
       </c>
-      <c r="S2" s="11" t="s">
-        <v>370</v>
-      </c>
-      <c r="T2" s="10" t="s">
+      <c r="Y1" s="8" t="s">
+        <v>367</v>
+      </c>
+      <c r="Z1" s="8" t="s">
         <v>368</v>
       </c>
-      <c r="U2" s="10" t="s">
+      <c r="AA1" s="9" t="s">
         <v>369</v>
       </c>
-      <c r="V2" s="11" t="s">
-        <v>370</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="N1:P1"/>
-    <mergeCell ref="Q1:S1"/>
-    <mergeCell ref="T1:V1"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>